<commit_message>
np-Optimierung korrigiert: MoE->np=4, Dense->np=1; Configs, Registry, Excel, Doku aktualisiert
</commit_message>
<xml_diff>
--- a/doc-git/lmstudio_configs.xlsx
+++ b/doc-git/lmstudio_configs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J80"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -471,10 +471,15 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Empfohlene Slots</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Offload Ratio</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>System Prompt (Einleitung)</t>
         </is>
@@ -509,14 +514,16 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="n">
         <v>18</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J2" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Gemma-4-26B-A4B-it (Q3_K_S), a helpful agentic multimodal Large Language Model (LLM) trained by GoogleMind. 
 Capabilities: 
@@ -541,19 +548,18 @@
           <t>LFM2 MoE</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>6</v>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="I3" t="n">
+        <v>4</v>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|startoftext|&gt;&lt;|im_start|&gt;system
 You are lfm2-24b-a2b (Q4_K_M), a helpful agentic LLM model trained by Liquid AI. You can interact with a computer to solve tasks.
@@ -588,19 +594,18 @@
           <t>LFM2 MoE</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:q8_0 (disabled)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
         <v>6</v>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr">
+      <c r="I4" t="n">
+        <v>4</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|startoftext|&gt;&lt;|im_start|&gt;system
 You are LFM2-8B-A1B (UD-Q8_K_XL),  a helpful agentic hybrid Large Language Model (LLM) trained by Liquid AI. 
@@ -634,17 +639,15 @@
           <t>Qwen2.5 Dense (Coder)</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>K:q5_1 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen2.5-Coder-32B-Instruct (Q3_K_S), a helpful Large Language Model (LLM) trained by Alibaba. 
 You can interact with a computer to solve tasks.
@@ -659,25 +662,23 @@
           <t>essentialai/rnj-1</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>RNJ Dense</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>K:f16 / V:q8_0</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t xml:space="preserve">You are rnj-1 (Q8_0) a dense Large Language Modell (LLM) of 8 billion parameters trained from scratch by Essential AI.
 Note: essentialai/rnj-1 in LM Studio is the instruct variant of this model.
@@ -715,14 +716,16 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
         <v>18</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t xml:space="preserve">You are gemma-4-26B-A4B-it-qat-q4_0 (Q4_0), a helpful agentic multimodal Large Language Model (LLM) trained by GoogleMind. 
 Capabilities: 
@@ -737,7 +740,6 @@
           <t>google/gemma-4-26b-a4b-it</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Gemma-4 (26B)</t>
@@ -748,14 +750,12 @@
           <t>gemma4-26b-template_minijinja.jinja</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>18</v>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -786,12 +786,13 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="n">
         <v>24</v>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
+      <c r="I9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t xml:space="preserve">You are granite-4.0-h-tiny (Q8_0), a helpful Large Language Model (LLM) trained by IBM.
 Supported Languages: English, German, Spanish, French, etc.
@@ -841,12 +842,13 @@
           <t>K:q5_1 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t xml:space="preserve">You are granite-4.1-30b (Q3_K_S), a helpful Large Language Model (LLM) trained by IBM.
 Supported Languages: English, German, Spanish, French, etc.
@@ -888,18 +890,18 @@
           <t>granite-4.1-30b_template.jinja</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t xml:space="preserve">You are granite-4.1-8b (Q8_0), a helpful Large Language Model (LLM) model trained by IBM. 
 Supported Languages: English, German, Spanish, French and more.
@@ -937,7 +939,6 @@
           <t>Mellum2 MoE</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="n">
         <v>131072</v>
       </c>
@@ -946,14 +947,16 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="n">
         <v>16</v>
       </c>
       <c r="I12" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Mellum2-12B-A2.5B-Instruct-i (Q4_K_M), a helpful agentic coding Large Language Model (LLM) trained by JetBrain. 
 The model uses a Mixture-of-Experts architecture with 64 experts and activates 8 experts per token. It uses a combination of sliding-window and full attention layers, with a context length of 131,072 tokens.
@@ -978,19 +981,18 @@
           <t>Mellum2 MoE</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q8_0 (disabled)</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="n">
         <v>6</v>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
+      <c r="I13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Mellum2-12B-A2.5B-Thinking, a helpful post-trained reasoning-augmented assistant LLM model trained by JetBrains. 
 You can interact with a computer to solve tasks.
@@ -1026,17 +1028,15 @@
           <t>Qwen3.6 MoE (REAP)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen3.6-35B-REAP-Pruned-ratio-0.5 (Q4_K_M), a helpful agentic Large Language Model (LLM) trained by Qwen. 
 You can interact with a computer to solve tasks.
@@ -1060,19 +1060,18 @@
           <t>LFM2 MoE</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="n">
         <v>12</v>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
+      <c r="I15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t xml:space="preserve">You are lfm2-24b-a2b (Q4_K_M), a helpful agentic LLM model trained by Liquid AI. You can interact with a computer to solve tasks.
 You are a Mixture of Experts (MoE) model with 24 billion total and  2.3 billion active parameters per token.
@@ -1106,19 +1105,18 @@
           <t>LFM2 MoE</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:q8_0</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
         <v>4</v>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|startoftext|&gt;&lt;|im_start|&gt;system
 You are LFM2.5-8B-A1B (Q8_0), a helpful agentic hybrid Large Language Model (LLM) trained by Liquid AI. 
@@ -1152,15 +1150,13 @@
           <t>CodeGemma Dense</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
         <v>1</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t xml:space="preserve">You are codegemma-7b-it (Q8_0), a helpful coding Large Language Model (LLM) trained by GoogleMind. 
 You have a context length of 8192 token.
@@ -1185,13 +1181,10 @@
           <t>Falcon3 Dense</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t xml:space="preserve">You are alcon3-10B-Instruct- (IQ4_XS), a helpful agentic coding LLM model trained by  TII Technology Innovation Institute. 
 Features:
@@ -1220,15 +1213,13 @@
           <t>GPT-OSS Dense</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="n">
         <v>16</v>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
+      <c r="I19" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t xml:space="preserve">You are gpt-oss-20b (Q6_K), a helpful agentic LLM model trained by OpenAI. You are a Mixture-of-Experts (MoE) and reasoning model and capable of \"Chain of Thought“.
 You are natively capable of function calling, web browsing, Python code execution, and Structured Outputs.\n\ngpt-oss-20b is for local use cases and has 21B parameters with 3.6B active parameters.
@@ -1259,12 +1250,9 @@
           <t>granite-4.1-30b_template.jinja</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1282,7 +1270,6 @@
           <t>Mistral Dense</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="n">
         <v>98304</v>
       </c>
@@ -1291,12 +1278,13 @@
           <t>K:q5_1 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
         <v>1</v>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Ministral-3-14B-Instruct-2512 (Q6_K), a helpful agentic coding Large Language Model (LLM) trained by Mistral AI. 
 </t>
@@ -1319,13 +1307,10 @@
           <t>Qwen2.5 Dense (Coder)</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen2.5-Coder-7B, a helpful agentic LLM model trained by Qwen. You can interact with a computer to solve tasks.
 User for code generation, code reasoning and code fixing, Code Agents. mathematics and general competencies.
@@ -1350,13 +1335,10 @@
           <t>Qwen2.5 Dense (Math)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen2.5-Math-7B-Instruct, a helpful Large Language Model (LLM) trained by Qwen. You can interact with a computer to solve tasks.
 User for code generation, code reasoning and code fixing, Code Agents. mathematics and general competencies.
@@ -1380,7 +1362,6 @@
           <t>StarCoder2 Dense</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="n">
         <v>16384</v>
       </c>
@@ -1389,10 +1370,10 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t xml:space="preserve">You are starcoder2-15b-instruct-v0.1 (Q6_K), a helpful agentic coding Large Language Model (LLM) trained by BigCode. You can interact with a computer to solve tasks.
 StarCoder2-15B-Instruct-v0.1 is primarily finetuned for Python code generation tasks that can be verified through execution, which may lead to certain biases and limitations. 
@@ -1417,13 +1398,10 @@
           <t>Solar Dense</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t xml:space="preserve">You are solar-pro-preview-instruct (Q4_K_S), a helpful agentic coding Large Language Model (LLM) trained by Solar-Pro. 
 Solar Pro Preview is developed using an enhanced version of our previous depth up-scaling method, which scales a Phi-3-medium model with 14 billion parameters to 22 billion parameters, 
@@ -1439,13 +1417,11 @@
           <t>microsoft/phi-4</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>Phi-4 Dense</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="n">
         <v>16384</v>
       </c>
@@ -1454,10 +1430,10 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
+      <c r="I26" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|im_start|&gt;system&lt;|im_sep|&gt;
 You are Phi-4, a helpful agentic LLM model trained by Microsoft. 
@@ -1494,13 +1470,10 @@
           <t>Phi-4 Dense</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
+      <c r="I27" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|im_start|&gt;system&lt;|im_sep|&gt;
 You are Phi-4, a helpful agentic Large Language Model (LLM) trained by Microsoft. 
@@ -1537,17 +1510,15 @@
           <t>Phi-4 Dense</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:q5_1</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
+      <c r="I28" t="n">
+        <v>1</v>
+      </c>
+      <c r="K28" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|im_start|&gt;system&lt;|im_sep|&gt;
 You are Phi-4, a helpful agentic LLM model trained by Microsoft. 
@@ -1574,25 +1545,23 @@
           <t>mistralai/codestral-22b-v0.1</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>Mistral Dense (Coder)</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
         <v>1</v>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t xml:space="preserve">You are codestral-22b-v0.1 (IQ4_XS or Q4_K_S), a helpful agentic coding Large Language Model (LLM) trained by Mistral AI. 
 </t>
@@ -1615,13 +1584,10 @@
           <t>AceMath</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" t="inlineStr">
         <is>
           <t xml:space="preserve">You are AceMath-7B-Instruct (Q8_0), a helpful Large Language Model (LLM) trained by NVIDIA.
 You are developed from the Qwen2.5-Math-Base models, leveraging a multi-stage supervised fine-tuning (SFT) process.
@@ -1648,7 +1614,6 @@
           <t>CodeLlama Dense</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="n">
         <v>16384</v>
       </c>
@@ -1657,10 +1622,10 @@
           <t>K:q5_1</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
+      <c r="I31" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" t="inlineStr">
         <is>
           <t xml:space="preserve">You are CodeLlama-13B-Instruct (Q8_0), a helpful agentic coding LLM model trained by Meta. 
  This model is designed for general code synthesis and understanding
@@ -1693,7 +1658,6 @@
           <t>CodeLlama Dense</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="n">
         <v>16384</v>
       </c>
@@ -1702,10 +1666,10 @@
           <t>K:q5_1</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
+      <c r="I32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" t="inlineStr">
         <is>
           <t xml:space="preserve">You are CodeLlama-13B-Python-HF (Q6_K), a helpful agentic coding LLM model trained by Meta. 
 Intended Use Cases Code Llama and its variants is intended for  use in English and relevant programming languages. 
@@ -1753,14 +1717,16 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="n">
         <v>18</v>
       </c>
       <c r="I33" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Gemma-4-19B-A4B-it-REAP-i1 (IQ4_NL), a helpful agentic multimodal Large Language Model (LLM) trained by GoogleMind. 
 Capabilities: 
@@ -1798,14 +1764,16 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="n">
         <v>18</v>
       </c>
       <c r="I34" t="n">
-        <v>1</v>
-      </c>
-      <c r="J34" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Gemma-4-19B-A4B-it-REAP-i1 (IQ4_NL), a helpful agentic multimodal Large Language Model (LLM) trained by GoogleMind. 
 Capabilities: 
@@ -1843,14 +1811,16 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="n">
         <v>18</v>
       </c>
       <c r="I35" t="n">
-        <v>1</v>
-      </c>
-      <c r="J35" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Gemma-4-19B-A4B-it-REAP-i1 (Q4_K_S), a helpful agentic multimodal Large Language Model (LLM) trained by GoogleMind. 
 Capabilities: 
@@ -1875,19 +1845,18 @@
           <t>GLM MoE</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>K:q8_0 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="n">
         <v>24</v>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
+      <c r="I36" t="n">
+        <v>4</v>
+      </c>
+      <c r="K36" t="inlineStr">
         <is>
           <t xml:space="preserve">You are GLM-4.7-Flash-REAP-23B-A3B (i1-Q4_K_S) a helpful agentic multimodal Large Language Model (LLM) with 23 billion parameters trained by GLM. You can interact with a computer to solve tasks.
 you are a vision-language model optimized for local deployment and low-latency applications. 
@@ -1931,12 +1900,13 @@
           <t>K:q5_1 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="n">
         <v>1</v>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="inlineStr">
         <is>
           <t xml:space="preserve">You are granite-4.1-30b-i1 (Q3_K_S),, a helpful Large Language Model (LLM) trained by IBM.
 Supported Languages: English, German, Spanish, French and more.
@@ -1974,19 +1944,18 @@
           <t>LFM2 MoE</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="n">
         <v>4</v>
       </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr">
+      <c r="I38" t="n">
+        <v>4</v>
+      </c>
+      <c r="K38" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|startoftext|&gt;&lt;|im_start|&gt;system
 You are lfm2-24b-a2b (Q6_K), a helpful agentic Large Language Model (LLM) trained by Liquid AI. You can interact with a computer to solve tasks.
@@ -2021,13 +1990,10 @@
           <t>MiMo MoE (Vision)</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
+      <c r="I39" t="n">
+        <v>4</v>
+      </c>
+      <c r="K39" t="inlineStr">
         <is>
           <t xml:space="preserve">You are MiMo-VL-7B-SFT-2508, a helpful agentic LLM model trained by Xiaomi. You can interact with a computer to solve tasks.
 Thinking Control Feature
@@ -2061,13 +2027,10 @@
           <t>Pythia Dense</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr">
+      <c r="I40" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" t="inlineStr">
         <is>
           <t xml:space="preserve">You are pythia-12b (Q6_K), a helpful coding model published by ...  
 Pythia is a general large language model (LLM) with 12 billion parameters, but a context length of only 2048 token.
@@ -2092,13 +2055,10 @@
           <t>Pythia Dense</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr">
+      <c r="I41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr">
         <is>
           <t xml:space="preserve">You are pythia-12b.i1 (Q6_K), a helpful coding model published by ...  
 Pythia is a general large language model (LLM) with 12 billion parameters, but a context length of only 2048 token.
@@ -2123,7 +2083,6 @@
           <t>Qwen3 MoE (Coder)</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>98304</v>
       </c>
@@ -2132,14 +2091,16 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="n">
         <v>16</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
-      </c>
-      <c r="J42" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen3-Coder-REAP-25B-A3B (Q3_K_M), a helpful agentic coding Large Language Model (LLM) trained by Alibaba. 
 This model was created using REAP (Router-weighted Expert Activation Pruning) from base model Qwen3-Coder-30B-A3B-Instruct to compress the weights matrix from 30B to 25B parameters,  
@@ -2168,7 +2129,6 @@
           <t>Qwen3 MoE (Coder)</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
       <c r="E43" t="n">
         <v>98304</v>
       </c>
@@ -2177,14 +2137,16 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
         <v>16</v>
       </c>
       <c r="I43" t="n">
-        <v>1</v>
-      </c>
-      <c r="J43" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen3-Coder-REAP-25B-A3B.i1 (Q3_K_M), a helpful agentic coding Large Language Model (LLM) trained by Alibaba. 
 Here the -i1 variant is the dynamic weighted/imatrix quants of the static weights Qwen3.6-Coder-REAP-25B.
@@ -2214,7 +2176,6 @@
           <t>Qwen3.6 MoE (REAP)</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>98304</v>
       </c>
@@ -2223,14 +2184,16 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="n">
         <v>18</v>
       </c>
       <c r="I44" t="n">
-        <v>1</v>
-      </c>
-      <c r="J44" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen3.6-28B-REAP-i1 (IQ3_S), a helpful Large Language Model (LLM) trained by Alibaba. 
 Here the -i1 variant is the weighted/imatrix quants of the static weights Qwen3.6-28B.
@@ -2262,7 +2225,6 @@
           <t>Qwen3.6 MoE (REAP)</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>98304</v>
       </c>
@@ -2271,14 +2233,16 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="n">
         <v>18</v>
       </c>
       <c r="I45" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen3.6-28B-REAP-i1 (Q3_K_S), a helpful Large Language Model (LLM) trained by Alibaba. 
 Here the -i1 variant is the weighted/imatrix quants of the static weights Qwen3.6-28B.
@@ -2310,13 +2274,10 @@
           <t>WizardCoder Dense</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr">
+      <c r="I46" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" t="inlineStr">
         <is>
           <t xml:space="preserve">You are wizardcoder-python-13b-v1.0 (Q6_K-i1), a helpful coding model trained by nlpxucan / WizardLM . 
 Wizard Coder is a code generation model based on Code Llama, date 09/7/2023.
@@ -2341,17 +2302,15 @@
           <t>Python Coder (custom)</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>K:f16 (disabled) / V:q8_0</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr">
+      <c r="I47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Nerdsking-python-coder-7B-i (Q8_0_i), a helpful agentic coding Large Language Model (LLM) trained by Nerdsking. 
 </t>
@@ -2374,13 +2333,10 @@
           <t>Qwen2 Dense</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr"/>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr">
+      <c r="I48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen2-audio-7b, a helpful LLM model trained by Qwen. You can interact with a computer to solve tasks.
 Qwen2-Audio is capable of accepting various audio signal inputs and performing audio analysis or direct textual responses with regard to speech instructions. 
@@ -2407,17 +2363,15 @@
           <t>Qwen2 Dense</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr"/>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>K:f16 / V:f16</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr">
+      <c r="I49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen2-Audio, a SOTA small-scale multimodal model (AudioLM) that handles audio and text inputs, allowing you to have voice interactions without ASR modules. 
 Qwen2-Audio supports English, Chinese, and major European languages, and provides voice chat and audio analysis capabilities for local use cases like:
@@ -2445,13 +2399,10 @@
           <t>Numina Math</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr"/>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr">
+      <c r="I50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t xml:space="preserve">You are NuminaMath-7b-CoT (Q8), a helpful agentic model trained by Mistral AI. 
 Yuu are Capable of Chain of Thought (CoT). This model is a Step-1 fine-tuned version of deepseek-ai/deepseek-math-7b-base.
@@ -2475,7 +2426,6 @@
           <t>Qwen2.5 Dense (Coder)</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>98304</v>
       </c>
@@ -2484,12 +2434,13 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="n">
         <v>1</v>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen2.5-14B-Instruct (Q5_0), a helpful Large Language Model (LLM) trained by Alibaba. 
 You can interact with a computer to solve tasks.
@@ -2521,7 +2472,6 @@
           <t>Qwen2.5 Dense (Coder)</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr"/>
       <c r="E52" t="n">
         <v>65536</v>
       </c>
@@ -2530,12 +2480,13 @@
           <t>K:q5_1 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="n">
         <v>1</v>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
+      <c r="K52" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen2.5-14B-Instruct (Q6_0), a helpful Large Language Model (LLM) trained by Alibaba. 
 You can interact with a computer to solve tasks.
@@ -2567,13 +2518,10 @@
           <t>CodeLlama Dense</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr"/>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
-      <c r="I53" t="inlineStr"/>
-      <c r="J53" t="inlineStr">
+      <c r="I53" t="n">
+        <v>1</v>
+      </c>
+      <c r="K53" t="inlineStr">
         <is>
           <t xml:space="preserve">You are CodeLlama-13B-Instruct (Q6_K), a helpful agentic coding model trained by Meta. You can interact with a computer to solve tasks.
 </t>
@@ -2596,17 +2544,15 @@
           <t>CodeLlama Dense</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr"/>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr">
+      <c r="I54" t="n">
+        <v>1</v>
+      </c>
+      <c r="K54" t="inlineStr">
         <is>
           <t xml:space="preserve">You are CodeLlama-13B-Python (Q6_K), a helpful agentic coding Large Language Model (LLM) trained by Meta. 
 </t>
@@ -2629,17 +2575,15 @@
           <t>DeepSeek Dense (Coder)</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q4_1</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr">
+      <c r="I55" t="n">
+        <v>1</v>
+      </c>
+      <c r="K55" t="inlineStr">
         <is>
           <t xml:space="preserve">You are deepseek-coder-33B-instruct (Q3_K_S), a helpful agentic Large Language Model (LLM) with 6.7 billion parameters trained by DeepSeek.
 You can interact with a computer to solve tasks.
@@ -2663,17 +2607,15 @@
           <t>DeepSeek Dense (Coder)</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>K:f16 (disabled) / V:q8_0 (disabled)</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr">
+      <c r="I56" t="n">
+        <v>1</v>
+      </c>
+      <c r="K56" t="inlineStr">
         <is>
           <t xml:space="preserve">You are deepseek-coder-6.7B-instruct (Q8_0), a helpful agentic Large Language Model (LLM) with 6.7 billion parameters trained by DeepSeek.
 You can interact with a computer to solve tasks.
@@ -2697,13 +2639,9 @@
           <t>Pandalyst Dense</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr"/>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="I57" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2721,17 +2659,15 @@
           <t>Pandalyst Dense</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:q8_0</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr">
+      <c r="I58" t="n">
+        <v>1</v>
+      </c>
+      <c r="K58" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Pandalyst_13B_V1.0 (Q5_0), a helpful coding Large Language Model (LLM) published by Patreon/The Bloke and created by Yanzhao Zheng. 
 Pandalyst is a general large language model with 13 billion parameter specifically trained to process and analyze data using the Python Pandas library.
@@ -2759,17 +2695,15 @@
           <t>Pandalyst Dense</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr"/>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>K:q8_0 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr">
+      <c r="I59" t="n">
+        <v>1</v>
+      </c>
+      <c r="K59" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Pandalyst_13B_V1.0 (Q6_K), a helpful coding model published by Patreon/The Bloke and created by Yanzhao Zheng. 
 Pandalyst is a general large language model with 13 billion parameter specifically trained to process and analyze data using the Python Pandas library.
@@ -2797,17 +2731,15 @@
           <t>WizardCoder Dense</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr"/>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr">
+      <c r="I60" t="n">
+        <v>1</v>
+      </c>
+      <c r="K60" t="inlineStr">
         <is>
           <t xml:space="preserve">You are WizardCoder-Python-13B-V1.0 (Q6_K), a helpfulLarge Language Model (LLM) trained by WizardLM. 
 You can interact with a computer to solve tasks.
@@ -2831,19 +2763,18 @@
           <t>Falcon3 Dense</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="n">
         <v>1</v>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="J61" t="n">
+        <v>1</v>
+      </c>
+      <c r="K61" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Falcon3-10B-Instruct- (Q8_0), a helpful agentic coding Large Language Model (LLM)  trained by  TII Technology Innovation Institute. 
 Features:
@@ -2872,7 +2803,6 @@
           <t>Mistral Dense (Coder)</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr"/>
       <c r="E62" t="n">
         <v>98304</v>
       </c>
@@ -2881,12 +2811,13 @@
           <t>K:q5_1 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="n">
         <v>1</v>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="J62" t="n">
+        <v>1</v>
+      </c>
+      <c r="K62" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Devstral-Small-2-24B-Instruct-2512 (Q3_K_S), a helpful agentic coding Large Language Model (LLM) trained by Mistral AI. 
 </t>
@@ -2909,7 +2840,6 @@
           <t>ERNIE MoE</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr"/>
       <c r="E63" t="n">
         <v>131072</v>
       </c>
@@ -2918,14 +2848,16 @@
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
         <v>14</v>
       </c>
       <c r="I63" t="n">
-        <v>1</v>
-      </c>
-      <c r="J63" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J63" t="n">
+        <v>1</v>
+      </c>
+      <c r="K63" t="inlineStr">
         <is>
           <t xml:space="preserve">You are ERNIE-4.5-21B-A3B-PT (IQ4_NL), a helpful multimodal Large Language Model (LLM) from Baidu.
 Ernie is a medium-size Mixture-of-Experts (MoE) post-trained model, with 21B total and 3B activated parameters.
@@ -2954,19 +2886,18 @@
           <t>ERNIE MoE</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr"/>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
         <v>8</v>
       </c>
-      <c r="I64" t="inlineStr"/>
-      <c r="J64" t="inlineStr">
+      <c r="I64" t="n">
+        <v>4</v>
+      </c>
+      <c r="K64" t="inlineStr">
         <is>
           <t xml:space="preserve">You are ERNIE-4.5-21B-A3B-Thinking (IQ4_NL), a helpful multimodal Large Language Model (LLM)  from Baidu.
 Ernie is a medium-size Mixture-of-Experts (MoE) post-trained model, with 21B total and 3B activated parameters for each token.
@@ -2999,15 +2930,13 @@
           <t>FLUX Diffusion (Vision)</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>2048</v>
       </c>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
-      <c r="I65" t="inlineStr"/>
-      <c r="J65" t="inlineStr">
+      <c r="I65" t="n">
+        <v>1</v>
+      </c>
+      <c r="K65" t="inlineStr">
         <is>
           <t xml:space="preserve">Your are FLUX.2-klein-9B, a helpful Vision Language Model from 
 black-forest-labs.
@@ -3054,14 +2983,16 @@
           <t>K:q8_0 (disabled) / V:q5_1 (disabled)</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr"/>
       <c r="H66" t="n">
         <v>18</v>
       </c>
       <c r="I66" t="n">
-        <v>1</v>
-      </c>
-      <c r="J66" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J66" t="n">
+        <v>1</v>
+      </c>
+      <c r="K66" t="inlineStr">
         <is>
           <t xml:space="preserve">You are gemma-4-26B-A4B-it-UD (IQ3_S), a helpful agentic multimodal Large Language Model (LLM) trained by GoogleMind. 
 Capabilities: 
@@ -3086,17 +3017,15 @@
           <t>GLM Vision</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
-      <c r="I67" t="inlineStr"/>
-      <c r="J67" t="inlineStr">
+      <c r="I67" t="n">
+        <v>1</v>
+      </c>
+      <c r="K67" t="inlineStr">
         <is>
           <t xml:space="preserve">You are GLM-4.6v-flash (UD-Q6_K_XL), a helpful agentic multimodal Large Language Model (LLM) with 9 billion parameters trained by GLM. You can interact with a computer to solve tasks.
 you are a vision-language model optimized for local deployment and low-latency applications. 
@@ -3127,19 +3056,18 @@
           <t>GLM MoE</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G68" t="inlineStr"/>
       <c r="H68" t="n">
         <v>6</v>
       </c>
-      <c r="I68" t="inlineStr"/>
-      <c r="J68" t="inlineStr">
+      <c r="I68" t="n">
+        <v>4</v>
+      </c>
+      <c r="K68" t="inlineStr">
         <is>
           <t xml:space="preserve">You are GLM-4.7-Flash-REAP-23B-A3B a helpful agentic Large Language Model (LLM) with 23 billion parameters trained by GLM. 
 You can interact with a computer to solve tasks.
@@ -3171,19 +3099,18 @@
           <t>GPT-OSS Dense</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:q8_0 (disabled)</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
       <c r="H69" t="n">
         <v>16</v>
       </c>
-      <c r="I69" t="inlineStr"/>
-      <c r="J69" t="inlineStr">
+      <c r="I69" t="n">
+        <v>4</v>
+      </c>
+      <c r="K69" t="inlineStr">
         <is>
           <t xml:space="preserve">You are gpt-oss-20b (Q6_K), a helpful agentic LLM model trained by OpenAI. You are a Mixture-of-Experts (MoE) and reasoning model and capable of \"Chain of Thought“.
 You are natively capable of function calling, web browsing, Python code execution, and Structured Outputs.\n\ngpt-oss-20b is for local use cases and has 21B parameters with 3.6B active parameters.
@@ -3214,16 +3141,15 @@
           <t>granite-4.0-h-tiny_template.jinja</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>K:q8_0 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr">
+      <c r="I70" t="n">
+        <v>4</v>
+      </c>
+      <c r="K70" t="inlineStr">
         <is>
           <t xml:space="preserve">You are granite-4.0-h-tiny (UD-Q8_K_XL), a helpful hybrid long-context finetuned Mixture of Expert (MoE) Large Language Model (LLM) trained by IBM, containing 7 billion total and 1 billion active parameters.
 Supported Languages: English, German, Spanish, French, etc.
@@ -3264,16 +3190,15 @@
           <t>granite-4.1-30b_template.jinja</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
-      <c r="I71" t="inlineStr"/>
-      <c r="J71" t="inlineStr">
+      <c r="I71" t="n">
+        <v>1</v>
+      </c>
+      <c r="K71" t="inlineStr">
         <is>
           <t xml:space="preserve">You are granite-4.1-8b (Q6__K_XL), a helpful long context finetuned instruct LLM model trained by IBM. 
 Supported Languages: English, German, Spanish, French and more.
@@ -3313,16 +3238,15 @@
           <t>granite-4.1-30b_template.jinja</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>K:q8_0 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
-      <c r="I72" t="inlineStr"/>
-      <c r="J72" t="inlineStr">
+      <c r="I72" t="n">
+        <v>1</v>
+      </c>
+      <c r="K72" t="inlineStr">
         <is>
           <t xml:space="preserve">You are granite-4.1-8b (Q8_K_XL), a helpful long context finetuned instruct LLM model trained by IBM. 
 Supported Languages: English, German, Spanish, French and more.
@@ -3357,17 +3281,15 @@
           <t>JanusCoder Dense</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:q8_0</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
-      <c r="J73" t="inlineStr">
+      <c r="I73" t="n">
+        <v>1</v>
+      </c>
+      <c r="K73" t="inlineStr">
         <is>
           <t xml:space="preserve">You are JanusCoder-14B (Q5_K_M), a helpful agentic coding LLM model trained by Janus. 
 This model is built upon open-source language models as Qwen3-14B. 
@@ -3392,17 +3314,15 @@
           <t>JanusCoder Dense</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr"/>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:q8_0</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr">
+      <c r="I74" t="n">
+        <v>1</v>
+      </c>
+      <c r="K74" t="inlineStr">
         <is>
           <t xml:space="preserve">You are JanusCoder-14B (UD-Q5_K_XL), a helpful agentic coding Large Language Model (LLM) trained by Janus. 
 This model is built upon open-source language models as Qwen3-14B. 
@@ -3427,17 +3347,15 @@
           <t>LFM2 MoE</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr"/>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr">
+      <c r="I75" t="n">
+        <v>4</v>
+      </c>
+      <c r="K75" t="inlineStr">
         <is>
           <t xml:space="preserve">You are LFM2-8B-A1B (UD-Q8_K_XL), a helpful agentic hybrid LLM model trained by Liquid AI. 
 You are a Mixture of Experts (MoE) model with 8 billion passive and 1.5 b active parameters per token with extended pre-training and reinforcement learning.
@@ -3470,17 +3388,15 @@
           <t>MiMo MoE (Vision)</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr">
+      <c r="I76" t="n">
+        <v>4</v>
+      </c>
+      <c r="K76" t="inlineStr">
         <is>
           <t xml:space="preserve">You are MiMo-VL-7B-RL-2508, a helpful agentic LLM model trained by Xiaomi. You can interact with a computer to solve tasks.
 Das Modell ist ein multimodales Sprachmodell (Vision-Language Models), das Bilder und Videos verstehen und darüber reasoning (schlussfolgern) kann.
@@ -3523,7 +3439,6 @@
           <t>North-Mini Dense (Coder)</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" t="n">
         <v>98304</v>
       </c>
@@ -3532,14 +3447,16 @@
           <t>K:q8_0 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G77" t="inlineStr"/>
       <c r="H77" t="n">
         <v>16</v>
       </c>
       <c r="I77" t="n">
-        <v>1</v>
-      </c>
-      <c r="J77" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J77" t="n">
+        <v>1</v>
+      </c>
+      <c r="K77" t="inlineStr">
         <is>
           <t xml:space="preserve">You are North-Mini-Code-1.0 (Q3_K_M), a helpful agentic coding Large Language Model (LLM) trained by Cohere Labs. 
 North Mini Code is an open weights research release of a 30B-A3B (3B active) parameter model optimized for code generation, agentic software engineering, terminal tasks and high-quality code generation.
@@ -3567,19 +3484,18 @@
           <t>Phi-4 Dense</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr"/>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>K:q8_0 / V:q5_1</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" t="n">
         <v>1</v>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="J78" t="n">
+        <v>1</v>
+      </c>
+      <c r="K78" t="inlineStr">
         <is>
           <t xml:space="preserve">&lt;|im_start|&gt;system&lt;|im_sep|&gt;
 You are Phi-4, a helpful agentic Large Language Model (LLM)  trained by Microsoft. 
@@ -3616,17 +3532,15 @@
           <t>Qwen3 Dense</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr"/>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>K:q8_0 (disabled) / V:iq4_nl (disabled)</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr">
+      <c r="I79" t="n">
+        <v>1</v>
+      </c>
+      <c r="K79" t="inlineStr">
         <is>
           <t xml:space="preserve">You are qwen3.5-14b (UD-Q5_K_XL), a helpful agentic Large Language Model (LLM) trained by Qwen. You can interact with a computer to solve tasks.
 Features:
@@ -3652,7 +3566,6 @@
           <t>Qwen3.6 MoE (REAP)</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr"/>
       <c r="E80" t="n">
         <v>65536</v>
       </c>
@@ -3661,12 +3574,13 @@
           <t>K:q5_1 / V:iq4_nl</t>
         </is>
       </c>
-      <c r="G80" t="inlineStr"/>
-      <c r="H80" t="inlineStr"/>
       <c r="I80" t="n">
         <v>1</v>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="J80" t="n">
+        <v>1</v>
+      </c>
+      <c r="K80" t="inlineStr">
         <is>
           <t xml:space="preserve">You are Qwen3.6-27B (Q3_K_S), a helpful Large Language Model (LLM) trained by Alibaba. 
 You can interact with a computer to solve tasks.

</xml_diff>